<commit_message>
Todas as bases atualizadas com dados de 2023 1 semestre
</commit_message>
<xml_diff>
--- a/data-raw/base_completa.xlsx
+++ b/data-raw/base_completa.xlsx
@@ -468,10 +468,10 @@
         </is>
       </c>
       <c r="B2">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="C2">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="D2">
         <v>32</v>
@@ -534,46 +534,46 @@
         </is>
       </c>
       <c r="B3">
-        <v>142</v>
+        <v>282</v>
       </c>
       <c r="C3">
-        <v>135</v>
+        <v>261</v>
       </c>
       <c r="D3">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="E3">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="F3">
-        <v>575</v>
+        <v>1144</v>
       </c>
       <c r="G3">
-        <v>422</v>
+        <v>827</v>
       </c>
       <c r="H3">
-        <v>33095</v>
+        <v>67177</v>
       </c>
       <c r="I3">
-        <v>3366</v>
+        <v>7381</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L3">
-        <v>526</v>
+        <v>1699</v>
       </c>
       <c r="M3">
-        <v>7526</v>
+        <v>13992</v>
       </c>
       <c r="N3">
-        <v>7386</v>
+        <v>13923</v>
       </c>
       <c r="O3">
-        <v>2283</v>
+        <v>4307</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
@@ -618,10 +618,10 @@
         <v>878</v>
       </c>
       <c r="H4">
-        <v>70009</v>
+        <v>69671</v>
       </c>
       <c r="I4">
-        <v>7330</v>
+        <v>7416</v>
       </c>
       <c r="J4">
         <v>0</v>
@@ -666,46 +666,46 @@
         </is>
       </c>
       <c r="B5">
-        <v>147</v>
+        <v>323</v>
       </c>
       <c r="C5">
-        <v>140</v>
+        <v>313</v>
       </c>
       <c r="D5">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="E5">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="F5">
-        <v>677</v>
+        <v>1275</v>
       </c>
       <c r="G5">
-        <v>491</v>
+        <v>943</v>
       </c>
       <c r="H5">
-        <v>36335</v>
+        <v>73250</v>
       </c>
       <c r="I5">
-        <v>3872</v>
+        <v>9065</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="L5">
-        <v>507</v>
+        <v>1130</v>
       </c>
       <c r="M5">
-        <v>6907</v>
+        <v>13455</v>
       </c>
       <c r="N5">
-        <v>7065</v>
+        <v>13193</v>
       </c>
       <c r="O5">
-        <v>2037</v>
+        <v>4011</v>
       </c>
       <c r="P5" t="inlineStr">
         <is>
@@ -713,10 +713,10 @@
         </is>
       </c>
       <c r="R5">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="S5">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="T5">
         <v>1</v>
@@ -744,16 +744,16 @@
         <v>22</v>
       </c>
       <c r="F6">
-        <v>1507</v>
+        <v>1510</v>
       </c>
       <c r="G6">
-        <v>1119</v>
+        <v>1115</v>
       </c>
       <c r="H6">
-        <v>68422</v>
+        <v>68400</v>
       </c>
       <c r="I6">
-        <v>7476</v>
+        <v>7458</v>
       </c>
       <c r="J6">
         <v>0</v>
@@ -778,6 +778,18 @@
           <t>Capital</t>
         </is>
       </c>
+      <c r="R6">
+        <v>71</v>
+      </c>
+      <c r="S6">
+        <v>36</v>
+      </c>
+      <c r="T6">
+        <v>1</v>
+      </c>
+      <c r="U6">
+        <v>5</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -786,10 +798,10 @@
         </is>
       </c>
       <c r="B7">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C7">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="D7">
         <v>22</v>
@@ -852,46 +864,46 @@
         </is>
       </c>
       <c r="B8">
-        <v>128</v>
+        <v>238</v>
       </c>
       <c r="C8">
-        <v>118</v>
+        <v>225</v>
       </c>
       <c r="D8">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="E8">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="F8">
-        <v>582</v>
+        <v>1160</v>
       </c>
       <c r="G8">
-        <v>470</v>
+        <v>947</v>
       </c>
       <c r="H8">
-        <v>14108</v>
+        <v>27852</v>
       </c>
       <c r="I8">
-        <v>2798</v>
+        <v>6208</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="L8">
-        <v>427</v>
+        <v>831</v>
       </c>
       <c r="M8">
-        <v>5908</v>
+        <v>11378</v>
       </c>
       <c r="N8">
-        <v>4596</v>
+        <v>8923</v>
       </c>
       <c r="O8">
-        <v>1670</v>
+        <v>3277</v>
       </c>
       <c r="P8" t="inlineStr">
         <is>
@@ -936,10 +948,10 @@
         <v>978</v>
       </c>
       <c r="H9">
-        <v>26894</v>
+        <v>26760</v>
       </c>
       <c r="I9">
-        <v>6364</v>
+        <v>6398</v>
       </c>
       <c r="J9">
         <v>0</v>
@@ -984,28 +996,28 @@
         </is>
       </c>
       <c r="B10">
-        <v>188</v>
+        <v>352</v>
       </c>
       <c r="C10">
-        <v>173</v>
+        <v>327</v>
       </c>
       <c r="D10">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="E10">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="F10">
-        <v>734</v>
+        <v>1407</v>
       </c>
       <c r="G10">
-        <v>552</v>
+        <v>1073</v>
       </c>
       <c r="H10">
-        <v>14500</v>
+        <v>28681</v>
       </c>
       <c r="I10">
-        <v>3445</v>
+        <v>8198</v>
       </c>
       <c r="J10">
         <v>0</v>
@@ -1014,16 +1026,16 @@
         <v>3</v>
       </c>
       <c r="L10">
-        <v>422</v>
+        <v>879</v>
       </c>
       <c r="M10">
-        <v>6224</v>
+        <v>11732</v>
       </c>
       <c r="N10">
-        <v>4247</v>
+        <v>8193</v>
       </c>
       <c r="O10">
-        <v>2302</v>
+        <v>4129</v>
       </c>
       <c r="P10" t="inlineStr">
         <is>
@@ -1062,16 +1074,16 @@
         <v>11</v>
       </c>
       <c r="F11">
-        <v>1341</v>
+        <v>1391</v>
       </c>
       <c r="G11">
-        <v>1044</v>
+        <v>1091</v>
       </c>
       <c r="H11">
-        <v>26006</v>
+        <v>25986</v>
       </c>
       <c r="I11">
-        <v>6052</v>
+        <v>6054</v>
       </c>
       <c r="J11">
         <v>0</v>
@@ -1096,6 +1108,18 @@
           <t>Grande São Paulo</t>
         </is>
       </c>
+      <c r="R11">
+        <v>17</v>
+      </c>
+      <c r="S11">
+        <v>14</v>
+      </c>
+      <c r="T11">
+        <v>1</v>
+      </c>
+      <c r="U11">
+        <v>1</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1104,10 +1128,10 @@
         </is>
       </c>
       <c r="B12">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="C12">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="D12">
         <v>32</v>
@@ -1170,46 +1194,46 @@
         </is>
       </c>
       <c r="B13">
-        <v>423</v>
+        <v>839</v>
       </c>
       <c r="C13">
-        <v>397</v>
+        <v>801</v>
       </c>
       <c r="D13">
-        <v>29</v>
+        <v>48</v>
       </c>
       <c r="E13">
-        <v>31</v>
+        <v>50</v>
       </c>
       <c r="F13">
-        <v>1814</v>
+        <v>3701</v>
       </c>
       <c r="G13">
-        <v>1450</v>
+        <v>2886</v>
       </c>
       <c r="H13">
-        <v>10667</v>
+        <v>21979</v>
       </c>
       <c r="I13">
-        <v>1983</v>
+        <v>4424</v>
       </c>
       <c r="J13">
         <v>0</v>
       </c>
       <c r="K13">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="L13">
-        <v>1743</v>
+        <v>3365</v>
       </c>
       <c r="M13">
-        <v>23835</v>
+        <v>45538</v>
       </c>
       <c r="N13">
-        <v>15410</v>
+        <v>30258</v>
       </c>
       <c r="O13">
-        <v>11062</v>
+        <v>20260</v>
       </c>
       <c r="P13" t="inlineStr">
         <is>
@@ -1254,10 +1278,10 @@
         <v>2869</v>
       </c>
       <c r="H14">
-        <v>23114</v>
+        <v>22718</v>
       </c>
       <c r="I14">
-        <v>4980</v>
+        <v>5016</v>
       </c>
       <c r="J14">
         <v>0</v>
@@ -1302,46 +1326,46 @@
         </is>
       </c>
       <c r="B15">
-        <v>449</v>
+        <v>915</v>
       </c>
       <c r="C15">
-        <v>427</v>
+        <v>874</v>
       </c>
       <c r="D15">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="E15">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="F15">
-        <v>1993</v>
+        <v>3853</v>
       </c>
       <c r="G15">
-        <v>1555</v>
+        <v>3009</v>
       </c>
       <c r="H15">
-        <v>11272</v>
+        <v>21911</v>
       </c>
       <c r="I15">
-        <v>2370</v>
+        <v>5628</v>
       </c>
       <c r="J15">
         <v>0</v>
       </c>
       <c r="K15">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="L15">
-        <v>1561</v>
+        <v>3171</v>
       </c>
       <c r="M15">
-        <v>25704</v>
+        <v>48043</v>
       </c>
       <c r="N15">
-        <v>15739</v>
+        <v>30345</v>
       </c>
       <c r="O15">
-        <v>12288</v>
+        <v>22061</v>
       </c>
       <c r="P15" t="inlineStr">
         <is>
@@ -1380,16 +1404,16 @@
         <v>47</v>
       </c>
       <c r="F16">
-        <v>4241</v>
+        <v>4286</v>
       </c>
       <c r="G16">
-        <v>3234</v>
+        <v>3262</v>
       </c>
       <c r="H16">
-        <v>22176</v>
+        <v>22123</v>
       </c>
       <c r="I16">
-        <v>5046</v>
+        <v>5055</v>
       </c>
       <c r="J16">
         <v>0</v>
@@ -1414,6 +1438,18 @@
           <t>Interior</t>
         </is>
       </c>
+      <c r="R16">
+        <v>82</v>
+      </c>
+      <c r="S16">
+        <v>12</v>
+      </c>
+      <c r="T16">
+        <v>4</v>
+      </c>
+      <c r="U16">
+        <v>2</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1493,46 +1529,46 @@
         </is>
       </c>
       <c r="B18">
-        <v>93</v>
+        <v>176</v>
       </c>
       <c r="C18">
-        <v>86</v>
+        <v>167</v>
       </c>
       <c r="D18">
+        <v>7</v>
+      </c>
+      <c r="E18">
+        <v>7</v>
+      </c>
+      <c r="F18">
+        <v>370</v>
+      </c>
+      <c r="G18">
+        <v>275</v>
+      </c>
+      <c r="H18">
+        <v>2568</v>
+      </c>
+      <c r="I18">
+        <v>466</v>
+      </c>
+      <c r="J18">
+        <v>0</v>
+      </c>
+      <c r="K18">
         <v>4</v>
       </c>
-      <c r="E18">
-        <v>4</v>
-      </c>
-      <c r="F18">
-        <v>181</v>
-      </c>
-      <c r="G18">
-        <v>147</v>
-      </c>
-      <c r="H18">
-        <v>1180</v>
-      </c>
-      <c r="I18">
-        <v>208</v>
-      </c>
-      <c r="J18">
-        <v>0</v>
-      </c>
-      <c r="K18">
-        <v>3</v>
-      </c>
       <c r="L18">
-        <v>226</v>
+        <v>427</v>
       </c>
       <c r="M18">
-        <v>1834</v>
+        <v>3445</v>
       </c>
       <c r="N18">
-        <v>1367</v>
+        <v>2626</v>
       </c>
       <c r="O18">
-        <v>705</v>
+        <v>1257</v>
       </c>
       <c r="P18" t="inlineStr">
         <is>
@@ -1582,10 +1618,10 @@
         <v>230</v>
       </c>
       <c r="H19">
-        <v>2412</v>
+        <v>2361</v>
       </c>
       <c r="I19">
-        <v>455</v>
+        <v>462</v>
       </c>
       <c r="J19">
         <v>0</v>
@@ -1635,46 +1671,46 @@
         </is>
       </c>
       <c r="B20">
-        <v>72</v>
+        <v>160</v>
       </c>
       <c r="C20">
-        <v>69</v>
+        <v>154</v>
       </c>
       <c r="D20">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E20">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F20">
-        <v>211</v>
+        <v>398</v>
       </c>
       <c r="G20">
-        <v>173</v>
+        <v>304</v>
       </c>
       <c r="H20">
-        <v>1113</v>
+        <v>2240</v>
       </c>
       <c r="I20">
-        <v>167</v>
+        <v>402</v>
       </c>
       <c r="J20">
         <v>0</v>
       </c>
       <c r="K20">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L20">
-        <v>203</v>
+        <v>409</v>
       </c>
       <c r="M20">
-        <v>2153</v>
+        <v>3944</v>
       </c>
       <c r="N20">
-        <v>1383</v>
+        <v>2732</v>
       </c>
       <c r="O20">
-        <v>906</v>
+        <v>1512</v>
       </c>
       <c r="P20" t="inlineStr">
         <is>
@@ -1718,16 +1754,16 @@
         <v>8</v>
       </c>
       <c r="F21">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="G21">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="H21">
         <v>2280</v>
       </c>
       <c r="I21">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="J21">
         <v>0</v>
@@ -1757,6 +1793,18 @@
           <t>Deinter 01</t>
         </is>
       </c>
+      <c r="R21">
+        <v>9</v>
+      </c>
+      <c r="S21">
+        <v>3</v>
+      </c>
+      <c r="T21">
+        <v>0</v>
+      </c>
+      <c r="U21">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1836,46 +1884,46 @@
         </is>
       </c>
       <c r="B23">
-        <v>50</v>
+        <v>102</v>
       </c>
       <c r="C23">
-        <v>45</v>
+        <v>92</v>
       </c>
       <c r="D23">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E23">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F23">
-        <v>240</v>
+        <v>499</v>
       </c>
       <c r="G23">
-        <v>196</v>
+        <v>388</v>
       </c>
       <c r="H23">
-        <v>2426</v>
+        <v>4927</v>
       </c>
       <c r="I23">
-        <v>774</v>
+        <v>1737</v>
       </c>
       <c r="J23">
         <v>0</v>
       </c>
       <c r="K23">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L23">
-        <v>303</v>
+        <v>492</v>
       </c>
       <c r="M23">
-        <v>2908</v>
+        <v>5634</v>
       </c>
       <c r="N23">
-        <v>2304</v>
+        <v>4496</v>
       </c>
       <c r="O23">
-        <v>945</v>
+        <v>1748</v>
       </c>
       <c r="P23" t="inlineStr">
         <is>
@@ -1925,10 +1973,10 @@
         <v>408</v>
       </c>
       <c r="H24">
-        <v>5007</v>
+        <v>4939</v>
       </c>
       <c r="I24">
-        <v>1847</v>
+        <v>1848</v>
       </c>
       <c r="J24">
         <v>0</v>
@@ -1978,46 +2026,46 @@
         </is>
       </c>
       <c r="B25">
-        <v>62</v>
+        <v>135</v>
       </c>
       <c r="C25">
-        <v>59</v>
+        <v>129</v>
       </c>
       <c r="D25">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E25">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="F25">
-        <v>276</v>
+        <v>498</v>
       </c>
       <c r="G25">
-        <v>206</v>
+        <v>380</v>
       </c>
       <c r="H25">
-        <v>2379</v>
+        <v>4648</v>
       </c>
       <c r="I25">
-        <v>767</v>
+        <v>1843</v>
       </c>
       <c r="J25">
         <v>0</v>
       </c>
       <c r="K25">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L25">
-        <v>223</v>
+        <v>433</v>
       </c>
       <c r="M25">
-        <v>2887</v>
+        <v>5514</v>
       </c>
       <c r="N25">
-        <v>2127</v>
+        <v>4188</v>
       </c>
       <c r="O25">
-        <v>1179</v>
+        <v>2137</v>
       </c>
       <c r="P25" t="inlineStr">
         <is>
@@ -2061,16 +2109,16 @@
         <v>9</v>
       </c>
       <c r="F26">
-        <v>602</v>
+        <v>605</v>
       </c>
       <c r="G26">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="H26">
-        <v>4276</v>
+        <v>4261</v>
       </c>
       <c r="I26">
-        <v>1591</v>
+        <v>1596</v>
       </c>
       <c r="J26">
         <v>0</v>
@@ -2100,6 +2148,18 @@
           <t>Deinter 02</t>
         </is>
       </c>
+      <c r="R26">
+        <v>10</v>
+      </c>
+      <c r="S26">
+        <v>1</v>
+      </c>
+      <c r="T26">
+        <v>1</v>
+      </c>
+      <c r="U26">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2179,46 +2239,46 @@
         </is>
       </c>
       <c r="B28">
-        <v>62</v>
+        <v>126</v>
       </c>
       <c r="C28">
-        <v>61</v>
+        <v>125</v>
       </c>
       <c r="D28">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E28">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F28">
-        <v>273</v>
+        <v>533</v>
       </c>
       <c r="G28">
-        <v>210</v>
+        <v>401</v>
       </c>
       <c r="H28">
-        <v>1453</v>
+        <v>3072</v>
       </c>
       <c r="I28">
-        <v>220</v>
+        <v>502</v>
       </c>
       <c r="J28">
         <v>0</v>
       </c>
       <c r="K28">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L28">
-        <v>263</v>
+        <v>532</v>
       </c>
       <c r="M28">
-        <v>3649</v>
+        <v>7075</v>
       </c>
       <c r="N28">
-        <v>2307</v>
+        <v>4610</v>
       </c>
       <c r="O28">
-        <v>1667</v>
+        <v>3029</v>
       </c>
       <c r="P28" t="inlineStr">
         <is>
@@ -2268,10 +2328,10 @@
         <v>383</v>
       </c>
       <c r="H29">
-        <v>2931</v>
+        <v>2874</v>
       </c>
       <c r="I29">
-        <v>607</v>
+        <v>618</v>
       </c>
       <c r="J29">
         <v>0</v>
@@ -2321,46 +2381,46 @@
         </is>
       </c>
       <c r="B30">
-        <v>62</v>
+        <v>123</v>
       </c>
       <c r="C30">
-        <v>60</v>
+        <v>118</v>
       </c>
       <c r="D30">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="E30">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="F30">
-        <v>304</v>
+        <v>576</v>
       </c>
       <c r="G30">
-        <v>215</v>
+        <v>405</v>
       </c>
       <c r="H30">
-        <v>1534</v>
+        <v>2903</v>
       </c>
       <c r="I30">
-        <v>302</v>
+        <v>721</v>
       </c>
       <c r="J30">
         <v>0</v>
       </c>
       <c r="K30">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L30">
-        <v>212</v>
+        <v>509</v>
       </c>
       <c r="M30">
-        <v>3908</v>
+        <v>7522</v>
       </c>
       <c r="N30">
-        <v>2381</v>
+        <v>4575</v>
       </c>
       <c r="O30">
-        <v>1908</v>
+        <v>3686</v>
       </c>
       <c r="P30" t="inlineStr">
         <is>
@@ -2404,16 +2464,16 @@
         <v>6</v>
       </c>
       <c r="F31">
-        <v>594</v>
+        <v>601</v>
       </c>
       <c r="G31">
-        <v>433</v>
+        <v>439</v>
       </c>
       <c r="H31">
-        <v>2717</v>
+        <v>2705</v>
       </c>
       <c r="I31">
-        <v>595</v>
+        <v>602</v>
       </c>
       <c r="J31">
         <v>0</v>
@@ -2443,6 +2503,18 @@
           <t>Deinter 03</t>
         </is>
       </c>
+      <c r="R31">
+        <v>11</v>
+      </c>
+      <c r="S31">
+        <v>0</v>
+      </c>
+      <c r="T31">
+        <v>0</v>
+      </c>
+      <c r="U31">
+        <v>1</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2522,28 +2594,28 @@
         </is>
       </c>
       <c r="B33">
-        <v>26</v>
+        <v>50</v>
       </c>
       <c r="C33">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="D33">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E33">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F33">
-        <v>162</v>
+        <v>327</v>
       </c>
       <c r="G33">
-        <v>131</v>
+        <v>260</v>
       </c>
       <c r="H33">
-        <v>339</v>
+        <v>648</v>
       </c>
       <c r="I33">
-        <v>23</v>
+        <v>59</v>
       </c>
       <c r="J33">
         <v>0</v>
@@ -2552,16 +2624,16 @@
         <v>1</v>
       </c>
       <c r="L33">
-        <v>115</v>
+        <v>311</v>
       </c>
       <c r="M33">
-        <v>2459</v>
+        <v>4510</v>
       </c>
       <c r="N33">
-        <v>1299</v>
+        <v>2426</v>
       </c>
       <c r="O33">
-        <v>1499</v>
+        <v>2709</v>
       </c>
       <c r="P33" t="inlineStr">
         <is>
@@ -2611,10 +2683,10 @@
         <v>276</v>
       </c>
       <c r="H34">
-        <v>664</v>
+        <v>646</v>
       </c>
       <c r="I34">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="J34">
         <v>0</v>
@@ -2664,46 +2736,46 @@
         </is>
       </c>
       <c r="B35">
-        <v>24</v>
+        <v>56</v>
       </c>
       <c r="C35">
-        <v>23</v>
+        <v>54</v>
       </c>
       <c r="D35">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E35">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F35">
-        <v>164</v>
+        <v>313</v>
       </c>
       <c r="G35">
-        <v>132</v>
+        <v>250</v>
       </c>
       <c r="H35">
-        <v>299</v>
+        <v>632</v>
       </c>
       <c r="I35">
-        <v>41</v>
+        <v>88</v>
       </c>
       <c r="J35">
         <v>0</v>
       </c>
       <c r="K35">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L35">
-        <v>162</v>
+        <v>273</v>
       </c>
       <c r="M35">
-        <v>2692</v>
+        <v>4991</v>
       </c>
       <c r="N35">
-        <v>1368</v>
+        <v>2645</v>
       </c>
       <c r="O35">
-        <v>1525</v>
+        <v>2735</v>
       </c>
       <c r="P35" t="inlineStr">
         <is>
@@ -2747,16 +2819,16 @@
         <v>5</v>
       </c>
       <c r="F36">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="G36">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="H36">
-        <v>558</v>
+        <v>554</v>
       </c>
       <c r="I36">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="J36">
         <v>0</v>
@@ -2786,6 +2858,18 @@
           <t>Deinter 04</t>
         </is>
       </c>
+      <c r="R36">
+        <v>3</v>
+      </c>
+      <c r="S36">
+        <v>0</v>
+      </c>
+      <c r="T36">
+        <v>1</v>
+      </c>
+      <c r="U36">
+        <v>0</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2865,10 +2949,10 @@
         </is>
       </c>
       <c r="B38">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="C38">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="D38">
         <v>1</v>
@@ -2877,16 +2961,16 @@
         <v>1</v>
       </c>
       <c r="F38">
-        <v>149</v>
+        <v>298</v>
       </c>
       <c r="G38">
-        <v>122</v>
+        <v>231</v>
       </c>
       <c r="H38">
-        <v>253</v>
+        <v>488</v>
       </c>
       <c r="I38">
-        <v>30</v>
+        <v>70</v>
       </c>
       <c r="J38">
         <v>0</v>
@@ -2895,16 +2979,16 @@
         <v>0</v>
       </c>
       <c r="L38">
-        <v>92</v>
+        <v>195</v>
       </c>
       <c r="M38">
-        <v>2098</v>
+        <v>3931</v>
       </c>
       <c r="N38">
-        <v>1056</v>
+        <v>2045</v>
       </c>
       <c r="O38">
-        <v>1184</v>
+        <v>2142</v>
       </c>
       <c r="P38" t="inlineStr">
         <is>
@@ -2954,10 +3038,10 @@
         <v>260</v>
       </c>
       <c r="H39">
-        <v>605</v>
+        <v>609</v>
       </c>
       <c r="I39">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="J39">
         <v>0</v>
@@ -3007,10 +3091,10 @@
         </is>
       </c>
       <c r="B40">
-        <v>23</v>
+        <v>55</v>
       </c>
       <c r="C40">
-        <v>21</v>
+        <v>53</v>
       </c>
       <c r="D40">
         <v>2</v>
@@ -3019,34 +3103,34 @@
         <v>2</v>
       </c>
       <c r="F40">
-        <v>201</v>
+        <v>362</v>
       </c>
       <c r="G40">
-        <v>154</v>
+        <v>294</v>
       </c>
       <c r="H40">
-        <v>318</v>
+        <v>584</v>
       </c>
       <c r="I40">
-        <v>40</v>
+        <v>88</v>
       </c>
       <c r="J40">
         <v>0</v>
       </c>
       <c r="K40">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L40">
-        <v>119</v>
+        <v>217</v>
       </c>
       <c r="M40">
-        <v>2301</v>
+        <v>4276</v>
       </c>
       <c r="N40">
-        <v>1154</v>
+        <v>2204</v>
       </c>
       <c r="O40">
-        <v>1292</v>
+        <v>2349</v>
       </c>
       <c r="P40" t="inlineStr">
         <is>
@@ -3093,13 +3177,13 @@
         <v>389</v>
       </c>
       <c r="G41">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="H41">
-        <v>522</v>
+        <v>518</v>
       </c>
       <c r="I41">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J41">
         <v>0</v>
@@ -3129,6 +3213,18 @@
           <t>Deinter 05</t>
         </is>
       </c>
+      <c r="R41">
+        <v>4</v>
+      </c>
+      <c r="S41">
+        <v>1</v>
+      </c>
+      <c r="T41">
+        <v>0</v>
+      </c>
+      <c r="U41">
+        <v>0</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -3137,10 +3233,10 @@
         </is>
       </c>
       <c r="B42">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C42">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D42">
         <v>2</v>
@@ -3208,28 +3304,28 @@
         </is>
       </c>
       <c r="B43">
-        <v>42</v>
+        <v>73</v>
       </c>
       <c r="C43">
-        <v>39</v>
+        <v>70</v>
       </c>
       <c r="D43">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E43">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F43">
-        <v>161</v>
+        <v>351</v>
       </c>
       <c r="G43">
-        <v>126</v>
+        <v>278</v>
       </c>
       <c r="H43">
-        <v>2833</v>
+        <v>5522</v>
       </c>
       <c r="I43">
-        <v>227</v>
+        <v>449</v>
       </c>
       <c r="J43">
         <v>0</v>
@@ -3238,16 +3334,16 @@
         <v>1</v>
       </c>
       <c r="L43">
-        <v>180</v>
+        <v>327</v>
       </c>
       <c r="M43">
-        <v>2288</v>
+        <v>4270</v>
       </c>
       <c r="N43">
-        <v>1516</v>
+        <v>2971</v>
       </c>
       <c r="O43">
-        <v>959</v>
+        <v>1714</v>
       </c>
       <c r="P43" t="inlineStr">
         <is>
@@ -3297,10 +3393,10 @@
         <v>263</v>
       </c>
       <c r="H44">
-        <v>6211</v>
+        <v>6158</v>
       </c>
       <c r="I44">
-        <v>449</v>
+        <v>458</v>
       </c>
       <c r="J44">
         <v>0</v>
@@ -3350,46 +3446,46 @@
         </is>
       </c>
       <c r="B45">
-        <v>49</v>
+        <v>93</v>
       </c>
       <c r="C45">
-        <v>47</v>
+        <v>90</v>
       </c>
       <c r="D45">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E45">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F45">
-        <v>157</v>
+        <v>345</v>
       </c>
       <c r="G45">
-        <v>119</v>
+        <v>262</v>
       </c>
       <c r="H45">
-        <v>3027</v>
+        <v>6160</v>
       </c>
       <c r="I45">
-        <v>307</v>
+        <v>640</v>
       </c>
       <c r="J45">
         <v>0</v>
       </c>
       <c r="K45">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L45">
-        <v>158</v>
+        <v>333</v>
       </c>
       <c r="M45">
-        <v>2193</v>
+        <v>4157</v>
       </c>
       <c r="N45">
-        <v>1645</v>
+        <v>3018</v>
       </c>
       <c r="O45">
-        <v>901</v>
+        <v>1636</v>
       </c>
       <c r="P45" t="inlineStr">
         <is>
@@ -3433,16 +3529,16 @@
         <v>6</v>
       </c>
       <c r="F46">
-        <v>395</v>
+        <v>414</v>
       </c>
       <c r="G46">
-        <v>298</v>
+        <v>314</v>
       </c>
       <c r="H46">
-        <v>7388</v>
+        <v>7385</v>
       </c>
       <c r="I46">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="J46">
         <v>0</v>
@@ -3472,6 +3568,18 @@
           <t>Deinter 06</t>
         </is>
       </c>
+      <c r="R46">
+        <v>18</v>
+      </c>
+      <c r="S46">
+        <v>3</v>
+      </c>
+      <c r="T46">
+        <v>0</v>
+      </c>
+      <c r="U46">
+        <v>0</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3551,46 +3659,46 @@
         </is>
       </c>
       <c r="B48">
-        <v>35</v>
+        <v>71</v>
       </c>
       <c r="C48">
-        <v>33</v>
+        <v>68</v>
       </c>
       <c r="D48">
+        <v>5</v>
+      </c>
+      <c r="E48">
+        <v>5</v>
+      </c>
+      <c r="F48">
+        <v>662</v>
+      </c>
+      <c r="G48">
+        <v>537</v>
+      </c>
+      <c r="H48">
+        <v>1624</v>
+      </c>
+      <c r="I48">
+        <v>309</v>
+      </c>
+      <c r="J48">
+        <v>0</v>
+      </c>
+      <c r="K48">
         <v>3</v>
       </c>
-      <c r="E48">
-        <v>3</v>
-      </c>
-      <c r="F48">
-        <v>319</v>
-      </c>
-      <c r="G48">
-        <v>259</v>
-      </c>
-      <c r="H48">
-        <v>741</v>
-      </c>
-      <c r="I48">
-        <v>143</v>
-      </c>
-      <c r="J48">
-        <v>0</v>
-      </c>
-      <c r="K48">
-        <v>2</v>
-      </c>
       <c r="L48">
-        <v>195</v>
+        <v>380</v>
       </c>
       <c r="M48">
-        <v>3217</v>
+        <v>6279</v>
       </c>
       <c r="N48">
-        <v>1890</v>
+        <v>3816</v>
       </c>
       <c r="O48">
-        <v>1715</v>
+        <v>3156</v>
       </c>
       <c r="P48" t="inlineStr">
         <is>
@@ -3640,10 +3748,10 @@
         <v>505</v>
       </c>
       <c r="H49">
-        <v>1815</v>
+        <v>1757</v>
       </c>
       <c r="I49">
-        <v>377</v>
+        <v>370</v>
       </c>
       <c r="J49">
         <v>0</v>
@@ -3693,46 +3801,46 @@
         </is>
       </c>
       <c r="B50">
-        <v>61</v>
+        <v>103</v>
       </c>
       <c r="C50">
-        <v>59</v>
+        <v>97</v>
       </c>
       <c r="D50">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E50">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F50">
-        <v>329</v>
+        <v>650</v>
       </c>
       <c r="G50">
-        <v>276</v>
+        <v>541</v>
       </c>
       <c r="H50">
-        <v>943</v>
+        <v>1740</v>
       </c>
       <c r="I50">
-        <v>189</v>
+        <v>495</v>
       </c>
       <c r="J50">
         <v>0</v>
       </c>
       <c r="K50">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L50">
-        <v>186</v>
+        <v>360</v>
       </c>
       <c r="M50">
-        <v>3583</v>
+        <v>6749</v>
       </c>
       <c r="N50">
-        <v>2000</v>
+        <v>3892</v>
       </c>
       <c r="O50">
-        <v>1832</v>
+        <v>3179</v>
       </c>
       <c r="P50" t="inlineStr">
         <is>
@@ -3776,16 +3884,16 @@
         <v>1</v>
       </c>
       <c r="F51">
-        <v>758</v>
+        <v>763</v>
       </c>
       <c r="G51">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="H51">
-        <v>1636</v>
+        <v>1631</v>
       </c>
       <c r="I51">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="J51">
         <v>0</v>
@@ -3815,6 +3923,18 @@
           <t>Deinter 07</t>
         </is>
       </c>
+      <c r="R51">
+        <v>5</v>
+      </c>
+      <c r="S51">
+        <v>2</v>
+      </c>
+      <c r="T51">
+        <v>2</v>
+      </c>
+      <c r="U51">
+        <v>0</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3894,28 +4014,28 @@
         </is>
       </c>
       <c r="B53">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="C53">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="D53">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E53">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F53">
-        <v>91</v>
+        <v>196</v>
       </c>
       <c r="G53">
-        <v>75</v>
+        <v>156</v>
       </c>
       <c r="H53">
-        <v>88</v>
+        <v>184</v>
       </c>
       <c r="I53">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="J53">
         <v>0</v>
@@ -3924,16 +4044,16 @@
         <v>0</v>
       </c>
       <c r="L53">
-        <v>93</v>
+        <v>152</v>
       </c>
       <c r="M53">
-        <v>1442</v>
+        <v>2844</v>
       </c>
       <c r="N53">
-        <v>782</v>
+        <v>1577</v>
       </c>
       <c r="O53">
-        <v>850</v>
+        <v>1641</v>
       </c>
       <c r="P53" t="inlineStr">
         <is>
@@ -3983,10 +4103,10 @@
         <v>135</v>
       </c>
       <c r="H54">
-        <v>218</v>
+        <v>208</v>
       </c>
       <c r="I54">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="J54">
         <v>0</v>
@@ -4036,10 +4156,10 @@
         </is>
       </c>
       <c r="B55">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="C55">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="D55">
         <v>0</v>
@@ -4048,16 +4168,16 @@
         <v>0</v>
       </c>
       <c r="F55">
-        <v>87</v>
+        <v>194</v>
       </c>
       <c r="G55">
-        <v>73</v>
+        <v>167</v>
       </c>
       <c r="H55">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="I55">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="J55">
         <v>0</v>
@@ -4066,16 +4186,16 @@
         <v>0</v>
       </c>
       <c r="L55">
-        <v>72</v>
+        <v>159</v>
       </c>
       <c r="M55">
-        <v>1691</v>
+        <v>3136</v>
       </c>
       <c r="N55">
-        <v>840</v>
+        <v>1603</v>
       </c>
       <c r="O55">
-        <v>1042</v>
+        <v>1884</v>
       </c>
       <c r="P55" t="inlineStr">
         <is>
@@ -4119,13 +4239,13 @@
         <v>1</v>
       </c>
       <c r="F56">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="G56">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H56">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="I56">
         <v>16</v>
@@ -4158,6 +4278,18 @@
           <t>Deinter 08</t>
         </is>
       </c>
+      <c r="R56">
+        <v>5</v>
+      </c>
+      <c r="S56">
+        <v>0</v>
+      </c>
+      <c r="T56">
+        <v>0</v>
+      </c>
+      <c r="U56">
+        <v>0</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -4237,10 +4369,10 @@
         </is>
       </c>
       <c r="B58">
-        <v>56</v>
+        <v>120</v>
       </c>
       <c r="C58">
-        <v>53</v>
+        <v>113</v>
       </c>
       <c r="D58">
         <v>3</v>
@@ -4249,34 +4381,34 @@
         <v>3</v>
       </c>
       <c r="F58">
-        <v>181</v>
+        <v>350</v>
       </c>
       <c r="G58">
-        <v>141</v>
+        <v>275</v>
       </c>
       <c r="H58">
-        <v>1202</v>
+        <v>2641</v>
       </c>
       <c r="I58">
-        <v>344</v>
+        <v>798</v>
       </c>
       <c r="J58">
         <v>0</v>
       </c>
       <c r="K58">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L58">
-        <v>195</v>
+        <v>398</v>
       </c>
       <c r="M58">
-        <v>2949</v>
+        <v>5671</v>
       </c>
       <c r="N58">
-        <v>2249</v>
+        <v>4481</v>
       </c>
       <c r="O58">
-        <v>1113</v>
+        <v>2055</v>
       </c>
       <c r="P58" t="inlineStr">
         <is>
@@ -4326,10 +4458,10 @@
         <v>281</v>
       </c>
       <c r="H59">
-        <v>2946</v>
+        <v>2864</v>
       </c>
       <c r="I59">
-        <v>1067</v>
+        <v>1071</v>
       </c>
       <c r="J59">
         <v>0</v>
@@ -4379,28 +4511,28 @@
         </is>
       </c>
       <c r="B60">
-        <v>64</v>
+        <v>110</v>
       </c>
       <c r="C60">
-        <v>58</v>
+        <v>102</v>
       </c>
       <c r="D60">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E60">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F60">
-        <v>194</v>
+        <v>367</v>
       </c>
       <c r="G60">
-        <v>151</v>
+        <v>284</v>
       </c>
       <c r="H60">
-        <v>1465</v>
+        <v>2625</v>
       </c>
       <c r="I60">
-        <v>543</v>
+        <v>1301</v>
       </c>
       <c r="J60">
         <v>0</v>
@@ -4409,16 +4541,16 @@
         <v>1</v>
       </c>
       <c r="L60">
-        <v>166</v>
+        <v>353</v>
       </c>
       <c r="M60">
-        <v>3233</v>
+        <v>5875</v>
       </c>
       <c r="N60">
-        <v>2251</v>
+        <v>4338</v>
       </c>
       <c r="O60">
-        <v>1177</v>
+        <v>2104</v>
       </c>
       <c r="P60" t="inlineStr">
         <is>
@@ -4462,16 +4594,16 @@
         <v>3</v>
       </c>
       <c r="F61">
-        <v>425</v>
+        <v>434</v>
       </c>
       <c r="G61">
-        <v>326</v>
+        <v>330</v>
       </c>
       <c r="H61">
-        <v>2444</v>
+        <v>2438</v>
       </c>
       <c r="I61">
-        <v>1269</v>
+        <v>1263</v>
       </c>
       <c r="J61">
         <v>0</v>
@@ -4501,6 +4633,18 @@
           <t>Deinter 09</t>
         </is>
       </c>
+      <c r="R61">
+        <v>14</v>
+      </c>
+      <c r="S61">
+        <v>1</v>
+      </c>
+      <c r="T61">
+        <v>0</v>
+      </c>
+      <c r="U61">
+        <v>1</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -4580,46 +4724,46 @@
         </is>
       </c>
       <c r="B63">
-        <v>22</v>
+        <v>48</v>
       </c>
       <c r="C63">
-        <v>19</v>
+        <v>45</v>
       </c>
       <c r="D63">
+        <v>3</v>
+      </c>
+      <c r="E63">
+        <v>4</v>
+      </c>
+      <c r="F63">
+        <v>115</v>
+      </c>
+      <c r="G63">
+        <v>85</v>
+      </c>
+      <c r="H63">
+        <v>305</v>
+      </c>
+      <c r="I63">
+        <v>21</v>
+      </c>
+      <c r="J63">
+        <v>0</v>
+      </c>
+      <c r="K63">
         <v>2</v>
       </c>
-      <c r="E63">
-        <v>3</v>
-      </c>
-      <c r="F63">
-        <v>57</v>
-      </c>
-      <c r="G63">
-        <v>43</v>
-      </c>
-      <c r="H63">
-        <v>152</v>
-      </c>
-      <c r="I63">
-        <v>10</v>
-      </c>
-      <c r="J63">
-        <v>0</v>
-      </c>
-      <c r="K63">
-        <v>0</v>
-      </c>
       <c r="L63">
-        <v>81</v>
+        <v>151</v>
       </c>
       <c r="M63">
-        <v>991</v>
+        <v>1879</v>
       </c>
       <c r="N63">
-        <v>640</v>
+        <v>1210</v>
       </c>
       <c r="O63">
-        <v>425</v>
+        <v>809</v>
       </c>
       <c r="P63" t="inlineStr">
         <is>
@@ -4669,10 +4813,10 @@
         <v>128</v>
       </c>
       <c r="H64">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="I64">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J64">
         <v>0</v>
@@ -4722,28 +4866,28 @@
         </is>
       </c>
       <c r="B65">
-        <v>17</v>
+        <v>40</v>
       </c>
       <c r="C65">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="D65">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E65">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F65">
-        <v>70</v>
+        <v>150</v>
       </c>
       <c r="G65">
-        <v>56</v>
+        <v>122</v>
       </c>
       <c r="H65">
-        <v>111</v>
+        <v>206</v>
       </c>
       <c r="I65">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="J65">
         <v>0</v>
@@ -4752,16 +4896,16 @@
         <v>0</v>
       </c>
       <c r="L65">
-        <v>60</v>
+        <v>125</v>
       </c>
       <c r="M65">
-        <v>1063</v>
+        <v>1879</v>
       </c>
       <c r="N65">
-        <v>590</v>
+        <v>1150</v>
       </c>
       <c r="O65">
-        <v>526</v>
+        <v>839</v>
       </c>
       <c r="P65" t="inlineStr">
         <is>
@@ -4805,16 +4949,16 @@
         <v>3</v>
       </c>
       <c r="F66">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="G66">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="H66">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="I66">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="J66">
         <v>0</v>
@@ -4844,6 +4988,18 @@
           <t>Deinter 10</t>
         </is>
       </c>
+      <c r="R66">
+        <v>3</v>
+      </c>
+      <c r="S66">
+        <v>1</v>
+      </c>
+      <c r="T66">
+        <v>0</v>
+      </c>
+      <c r="U66">
+        <v>0</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -4852,10 +5008,10 @@
         </is>
       </c>
       <c r="B67">
-        <v>1486</v>
+        <v>1482</v>
       </c>
       <c r="C67">
-        <v>1424</v>
+        <v>1421</v>
       </c>
       <c r="D67">
         <v>86</v>
@@ -4918,46 +5074,46 @@
         </is>
       </c>
       <c r="B68">
-        <v>693</v>
+        <v>1359</v>
       </c>
       <c r="C68">
-        <v>650</v>
+        <v>1287</v>
       </c>
       <c r="D68">
-        <v>45</v>
+        <v>80</v>
       </c>
       <c r="E68">
-        <v>48</v>
+        <v>85</v>
       </c>
       <c r="F68">
-        <v>2971</v>
+        <v>6005</v>
       </c>
       <c r="G68">
-        <v>2342</v>
+        <v>4660</v>
       </c>
       <c r="H68">
-        <v>57870</v>
+        <v>117008</v>
       </c>
       <c r="I68">
-        <v>8147</v>
+        <v>18013</v>
       </c>
       <c r="J68">
         <v>0</v>
       </c>
       <c r="K68">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="L68">
-        <v>2696</v>
+        <v>5895</v>
       </c>
       <c r="M68">
-        <v>37269</v>
+        <v>70908</v>
       </c>
       <c r="N68">
-        <v>27392</v>
+        <v>53104</v>
       </c>
       <c r="O68">
-        <v>15015</v>
+        <v>27844</v>
       </c>
       <c r="P68" t="inlineStr">
         <is>
@@ -5002,10 +5158,10 @@
         <v>4725</v>
       </c>
       <c r="H69">
-        <v>120017</v>
+        <v>119149</v>
       </c>
       <c r="I69">
-        <v>18674</v>
+        <v>18830</v>
       </c>
       <c r="J69">
         <v>0</v>
@@ -5050,46 +5206,46 @@
         </is>
       </c>
       <c r="B70">
-        <v>784</v>
+        <v>1590</v>
       </c>
       <c r="C70">
-        <v>740</v>
+        <v>1514</v>
       </c>
       <c r="D70">
-        <v>39</v>
+        <v>93</v>
       </c>
       <c r="E70">
-        <v>39</v>
+        <v>93</v>
       </c>
       <c r="F70">
-        <v>3404</v>
+        <v>6535</v>
       </c>
       <c r="G70">
-        <v>2598</v>
+        <v>5025</v>
       </c>
       <c r="H70">
-        <v>62107</v>
+        <v>123842</v>
       </c>
       <c r="I70">
-        <v>9687</v>
+        <v>22891</v>
       </c>
       <c r="J70">
         <v>0</v>
       </c>
       <c r="K70">
-        <v>21</v>
+        <v>41</v>
       </c>
       <c r="L70">
-        <v>2490</v>
+        <v>5180</v>
       </c>
       <c r="M70">
-        <v>38835</v>
+        <v>73230</v>
       </c>
       <c r="N70">
-        <v>27051</v>
+        <v>51731</v>
       </c>
       <c r="O70">
-        <v>16627</v>
+        <v>30201</v>
       </c>
       <c r="P70" t="inlineStr">
         <is>
@@ -5097,10 +5253,10 @@
         </is>
       </c>
       <c r="R70">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="S70">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="T70">
         <v>3</v>
@@ -5128,16 +5284,16 @@
         <v>80</v>
       </c>
       <c r="F71">
-        <v>7089</v>
+        <v>7187</v>
       </c>
       <c r="G71">
-        <v>5397</v>
+        <v>5468</v>
       </c>
       <c r="H71">
-        <v>116604</v>
+        <v>116509</v>
       </c>
       <c r="I71">
-        <v>18574</v>
+        <v>18567</v>
       </c>
       <c r="J71">
         <v>0</v>
@@ -5161,6 +5317,18 @@
         <is>
           <t>Estado de São Paulo</t>
         </is>
+      </c>
+      <c r="R71">
+        <v>170</v>
+      </c>
+      <c r="S71">
+        <v>62</v>
+      </c>
+      <c r="T71">
+        <v>6</v>
+      </c>
+      <c r="U71">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>